<commit_message>
Add invoice number per HS code to Kollmorgen CZ26016140 summary
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y21QzKwBo4M2zgxK76CjWb
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Kollmorgen_CZ26016140.xlsx
+++ b/output/HS_Code_Summary_Kollmorgen_CZ26016140.xlsx
@@ -469,19 +469,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="36" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="60" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -502,35 +503,40 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Faktura č.</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Země původu (COO)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Celkové množství (ks)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Čistá hmotnost (kg)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Hrubá hmotnost (kg)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Hodnota SEK – Total</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Příznak</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Poznámka</t>
         </is>
@@ -554,27 +560,32 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>5976477, 5976478</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
           <t>LT, SE, US</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="F2" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="F2" s="3" t="n">
+      <c r="G2" s="3" t="n">
         <v>46.63</v>
       </c>
-      <c r="G2" s="3" t="n">
+      <c r="H2" s="3" t="n">
         <v>77.95399999999999</v>
       </c>
-      <c r="H2" s="4" t="n">
+      <c r="I2" s="4" t="n">
         <v>128376</v>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>VÝVOZ</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Vč. příplatku za materiál 699 SEK (DN 5976478 ř. 9.1) k ř. 3.1 (83A21300A) – dle pokynu klienta vykázáno jako celek: 8537109199, 13 404 SEK, původ US.</t>
         </is>
@@ -598,27 +609,32 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
+          <t>5976477, 5976478</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
           <t>LT</t>
         </is>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="F3" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="F3" s="3" t="n">
+      <c r="G3" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="G3" s="3" t="n">
+      <c r="H3" s="3" t="n">
         <v>8.247</v>
       </c>
-      <c r="H3" s="4" t="n">
+      <c r="I3" s="4" t="n">
         <v>29255</v>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>VÝVOZ</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>Kód uveden klientem i na faktuře jen 8místně (KN).</t>
         </is>
@@ -642,27 +658,32 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
+          <t>5976477, 5976478</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
           <t>SE</t>
         </is>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="F4" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="F4" s="3" t="n">
+      <c r="G4" s="3" t="n">
         <v>0.9</v>
       </c>
-      <c r="G4" s="3" t="n">
+      <c r="H4" s="3" t="n">
         <v>1.508</v>
       </c>
-      <c r="H4" s="4" t="n">
+      <c r="I4" s="4" t="n">
         <v>4620</v>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>VÝVOZ</t>
         </is>
       </c>
-      <c r="J4" s="2" t="n"/>
+      <c r="K4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -682,27 +703,32 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
+          <t>5976477, 5976478</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
           <t>US</t>
         </is>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="F5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="F5" s="3" t="n">
+      <c r="G5" s="3" t="n">
         <v>0.49</v>
       </c>
-      <c r="G5" s="3" t="n">
+      <c r="H5" s="3" t="n">
         <v>0.822</v>
       </c>
-      <c r="H5" s="4" t="n">
+      <c r="I5" s="4" t="n">
         <v>2602</v>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>VÝVOZ</t>
         </is>
       </c>
-      <c r="J5" s="2" t="n"/>
+      <c r="K5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -722,27 +748,32 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
+          <t>5976477, 5976478</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
           <t>HU</t>
         </is>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="F6" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="F6" s="3" t="n">
+      <c r="G6" s="3" t="n">
         <v>0.28</v>
       </c>
-      <c r="G6" s="3" t="n">
+      <c r="H6" s="3" t="n">
         <v>0.469</v>
       </c>
-      <c r="H6" s="4" t="n">
+      <c r="I6" s="4" t="n">
         <v>316</v>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>VÝVOZ</t>
         </is>
       </c>
-      <c r="J6" s="2" t="n"/>
+      <c r="K6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -753,11 +784,8 @@
       <c r="B7" s="5" t="n"/>
       <c r="C7" s="5" t="n"/>
       <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5">
-        <f>SUM(E2:E6)</f>
-        <v/>
-      </c>
-      <c r="F7" s="6">
+      <c r="E7" s="5" t="n"/>
+      <c r="F7" s="5">
         <f>SUM(F2:F6)</f>
         <v/>
       </c>
@@ -765,12 +793,16 @@
         <f>SUM(G2:G6)</f>
         <v/>
       </c>
-      <c r="H7" s="7">
+      <c r="H7" s="6">
         <f>SUM(H2:H6)</f>
         <v/>
       </c>
-      <c r="I7" s="5" t="n"/>
+      <c r="I7" s="7">
+        <f>SUM(I2:I6)</f>
+        <v/>
+      </c>
       <c r="J7" s="5" t="n"/>
+      <c r="K7" s="5" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
@@ -898,17 +930,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -924,30 +957,35 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Faktura č.</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Země původu</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Množství (ks)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Čistá hmotnost (kg)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Hrubá hmotnost (kg)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Hodnota SEK – Total</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Řádky faktur (CI/ř.)</t>
         </is>
@@ -966,24 +1004,29 @@
       </c>
       <c r="C2" s="9" t="inlineStr">
         <is>
+          <t>5976477, 5976478</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
           <t>LT</t>
         </is>
       </c>
-      <c r="D2" s="9" t="n">
+      <c r="E2" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="E2" s="10" t="n">
+      <c r="F2" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="F2" s="10" t="n">
+      <c r="G2" s="10" t="n">
         <v>6.667</v>
       </c>
-      <c r="G2" s="11" t="n">
+      <c r="H2" s="11" t="n">
         <v>57165</v>
       </c>
-      <c r="H2" s="9" t="inlineStr">
-        <is>
-          <t>5976477/1.1, 5976478/1.1</t>
+      <c r="I2" s="9" t="inlineStr">
+        <is>
+          <t>5976477 ř. 1.1, 5976478 ř. 1.1</t>
         </is>
       </c>
     </row>
@@ -1000,24 +1043,29 @@
       </c>
       <c r="C3" s="9" t="inlineStr">
         <is>
+          <t>5976477, 5976478</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
           <t>SE</t>
         </is>
       </c>
-      <c r="D3" s="9" t="n">
+      <c r="E3" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="E3" s="10" t="n">
+      <c r="F3" s="10" t="n">
         <v>37.23</v>
       </c>
-      <c r="F3" s="10" t="n">
+      <c r="G3" s="10" t="n">
         <v>62.473</v>
       </c>
-      <c r="G3" s="11" t="n">
+      <c r="H3" s="11" t="n">
         <v>57807</v>
       </c>
-      <c r="H3" s="9" t="inlineStr">
-        <is>
-          <t>5976477/3.1, 5976477/4.1, 5976477/5.1, 5976478/4.1</t>
+      <c r="I3" s="9" t="inlineStr">
+        <is>
+          <t>5976477 ř. 3.1, 5976477 ř. 4.1, 5976477 ř. 5.1, 5976478 ř. 4.1</t>
         </is>
       </c>
     </row>
@@ -1034,24 +1082,29 @@
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
+          <t>5976478</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
           <t>US</t>
         </is>
       </c>
-      <c r="D4" s="9" t="n">
+      <c r="E4" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E4" s="10" t="n">
+      <c r="F4" s="10" t="n">
         <v>5.4</v>
       </c>
-      <c r="F4" s="10" t="n">
+      <c r="G4" s="10" t="n">
         <v>8.814</v>
       </c>
-      <c r="G4" s="11" t="n">
+      <c r="H4" s="11" t="n">
         <v>13404</v>
       </c>
-      <c r="H4" s="9" t="inlineStr">
-        <is>
-          <t>5976478/3.1, 5976478/9.1</t>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>5976478 ř. 3.1, 5976478 ř. 9.1</t>
         </is>
       </c>
     </row>
@@ -1068,24 +1121,29 @@
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
+          <t>5976477, 5976478</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
           <t>LT</t>
         </is>
       </c>
-      <c r="D5" s="9" t="n">
+      <c r="E5" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="E5" s="10" t="n">
+      <c r="F5" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="F5" s="10" t="n">
+      <c r="G5" s="10" t="n">
         <v>8.247</v>
       </c>
-      <c r="G5" s="11" t="n">
+      <c r="H5" s="11" t="n">
         <v>29255</v>
       </c>
-      <c r="H5" s="9" t="inlineStr">
-        <is>
-          <t>5976477/2.1, 5976478/2.1</t>
+      <c r="I5" s="9" t="inlineStr">
+        <is>
+          <t>5976477 ř. 2.1, 5976478 ř. 2.1</t>
         </is>
       </c>
     </row>
@@ -1102,24 +1160,29 @@
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
+          <t>5976477, 5976478</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
           <t>SE</t>
         </is>
       </c>
-      <c r="D6" s="9" t="n">
+      <c r="E6" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="E6" s="10" t="n">
+      <c r="F6" s="10" t="n">
         <v>0.9</v>
       </c>
-      <c r="F6" s="10" t="n">
+      <c r="G6" s="10" t="n">
         <v>1.508</v>
       </c>
-      <c r="G6" s="11" t="n">
+      <c r="H6" s="11" t="n">
         <v>4620</v>
       </c>
-      <c r="H6" s="9" t="inlineStr">
-        <is>
-          <t>5976477/6.1, 5976478/5.1</t>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>5976477 ř. 6.1, 5976478 ř. 5.1</t>
         </is>
       </c>
     </row>
@@ -1136,24 +1199,29 @@
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
+          <t>5976477, 5976478</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
           <t>US</t>
         </is>
       </c>
-      <c r="D7" s="9" t="n">
+      <c r="E7" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="E7" s="10" t="n">
+      <c r="F7" s="10" t="n">
         <v>0.49</v>
       </c>
-      <c r="F7" s="10" t="n">
+      <c r="G7" s="10" t="n">
         <v>0.822</v>
       </c>
-      <c r="G7" s="11" t="n">
+      <c r="H7" s="11" t="n">
         <v>2602</v>
       </c>
-      <c r="H7" s="9" t="inlineStr">
-        <is>
-          <t>5976477/7.1, 5976477/8.1, 5976478/6.1, 5976478/7.1</t>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>5976477 ř. 7.1, 5976477 ř. 8.1, 5976478 ř. 6.1, 5976478 ř. 7.1</t>
         </is>
       </c>
     </row>
@@ -1170,24 +1238,29 @@
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
+          <t>5976477, 5976478</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
           <t>HU</t>
         </is>
       </c>
-      <c r="D8" s="9" t="n">
+      <c r="E8" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E8" s="10" t="n">
+      <c r="F8" s="10" t="n">
         <v>0.28</v>
       </c>
-      <c r="F8" s="10" t="n">
+      <c r="G8" s="10" t="n">
         <v>0.469</v>
       </c>
-      <c r="G8" s="11" t="n">
+      <c r="H8" s="11" t="n">
         <v>316</v>
       </c>
-      <c r="H8" s="9" t="inlineStr">
-        <is>
-          <t>5976477/9.1, 5976478/8.1</t>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>5976477 ř. 9.1, 5976478 ř. 8.1</t>
         </is>
       </c>
     </row>
@@ -1199,11 +1272,8 @@
       </c>
       <c r="B9" s="5" t="n"/>
       <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5">
-        <f>SUM(D2:D8)</f>
-        <v/>
-      </c>
-      <c r="E9" s="6">
+      <c r="D9" s="5" t="n"/>
+      <c r="E9" s="5">
         <f>SUM(E2:E8)</f>
         <v/>
       </c>
@@ -1211,11 +1281,15 @@
         <f>SUM(F2:F8)</f>
         <v/>
       </c>
-      <c r="G9" s="7">
+      <c r="G9" s="6">
         <f>SUM(G2:G8)</f>
         <v/>
       </c>
-      <c r="H9" s="5" t="n"/>
+      <c r="H9" s="7">
+        <f>SUM(H2:H8)</f>
+        <v/>
+      </c>
+      <c r="I9" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>